<commit_message>
Update WTG acoustic spectra
</commit_message>
<xml_diff>
--- a/WTG_Acoustic_Spectra_Loudest_Modes 1.xlsx
+++ b/WTG_Acoustic_Spectra_Loudest_Modes 1.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{303D3440-1F9B-493C-86E1-A54AAFE94D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanking/Python/wind_noise_analyser/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DEFA41A-9E9C-774B-8906-03ABE1D5DB78}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Envision_EN182_N01_1-3oct" sheetId="1" r:id="rId1"/>
-    <sheet name="Nordex_N175_152m_ModeA_1-3oct" sheetId="2" r:id="rId2"/>
-    <sheet name="Siemens_SG7_AM0_1-1oct" sheetId="3" r:id="rId3"/>
+    <sheet name="Envision_EN182_N02 Serrations" sheetId="1" r:id="rId1"/>
+    <sheet name="GE 6.5-164" sheetId="4" r:id="rId2"/>
+    <sheet name="Nordex_N175_152m_ModeA_1-3oct" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -22,10 +27,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,22 +38,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
   <si>
     <t>Frequency_Hz</t>
   </si>
   <si>
     <t>Lw_dBA</t>
   </si>
-  <si>
-    <t>Octave_Centre_Frequency_Hz</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -61,13 +66,45 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="GE Inspira"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="GE Inspira Sans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="GE Inspira Sans"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -94,17 +131,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{6357D21A-838F-6046-BF44-C3FCF0B041FE}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -405,7 +451,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -416,227 +462,227 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>20</v>
       </c>
-      <c r="B2">
-        <v>68.5</v>
+      <c r="B2" s="2">
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>25</v>
       </c>
-      <c r="B3">
-        <v>70.8</v>
+      <c r="B3" s="2">
+        <v>69.3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>31.5</v>
       </c>
-      <c r="B4">
-        <v>73.5</v>
+      <c r="B4" s="2">
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>40</v>
       </c>
-      <c r="B5">
-        <v>76.7</v>
+      <c r="B5" s="2">
+        <v>75.2</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>50</v>
       </c>
-      <c r="B6">
-        <v>80.2</v>
+      <c r="B6" s="2">
+        <v>78.7</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>63</v>
       </c>
-      <c r="B7">
-        <v>84</v>
+      <c r="B7" s="2">
+        <v>82.5</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8">
+      <c r="A8" s="2">
         <v>80</v>
       </c>
-      <c r="B8">
-        <v>88.2</v>
+      <c r="B8" s="2">
+        <v>86.7</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>100</v>
       </c>
-      <c r="B9">
-        <v>92.1</v>
+      <c r="B9" s="2">
+        <v>90.6</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>125</v>
       </c>
-      <c r="B10">
-        <v>95.8</v>
+      <c r="B10" s="2">
+        <v>94.3</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>160</v>
       </c>
-      <c r="B11">
-        <v>99.4</v>
+      <c r="B11" s="2">
+        <v>97.9</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>200</v>
       </c>
-      <c r="B12">
-        <v>101.9</v>
+      <c r="B12" s="2">
+        <v>100.4</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13">
+      <c r="A13" s="2">
         <v>250</v>
       </c>
-      <c r="B13">
-        <v>103.6</v>
+      <c r="B13" s="2">
+        <v>102.1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14">
+      <c r="A14" s="2">
         <v>315</v>
       </c>
-      <c r="B14">
-        <v>104.6</v>
+      <c r="B14" s="2">
+        <v>103.1</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>400</v>
       </c>
-      <c r="B15">
-        <v>104.9</v>
+      <c r="B15" s="2">
+        <v>103.4</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>500</v>
       </c>
-      <c r="B16">
-        <v>104.7</v>
+      <c r="B16" s="2">
+        <v>103.2</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>630</v>
       </c>
-      <c r="B17">
-        <v>104.3</v>
+      <c r="B17" s="2">
+        <v>102.8</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18">
+      <c r="A18" s="2">
         <v>800</v>
       </c>
-      <c r="B18">
-        <v>103.6</v>
+      <c r="B18" s="2">
+        <v>102.1</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>1000</v>
       </c>
-      <c r="B19">
-        <v>102.7</v>
+      <c r="B19" s="2">
+        <v>101.2</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20">
+      <c r="A20" s="2">
         <v>1250</v>
       </c>
-      <c r="B20">
-        <v>101.6</v>
+      <c r="B20" s="2">
+        <v>100.1</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21">
+      <c r="A21" s="2">
         <v>1600</v>
       </c>
-      <c r="B21">
-        <v>100.2</v>
+      <c r="B21" s="2">
+        <v>98.7</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22">
+      <c r="A22" s="2">
         <v>2000</v>
       </c>
-      <c r="B22">
-        <v>98.5</v>
+      <c r="B22" s="2">
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23">
+      <c r="A23" s="2">
         <v>2500</v>
       </c>
-      <c r="B23">
-        <v>96.5</v>
+      <c r="B23" s="2">
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24">
+      <c r="A24" s="2">
         <v>3150</v>
       </c>
-      <c r="B24">
-        <v>94</v>
+      <c r="B24" s="2">
+        <v>92.5</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25">
+      <c r="A25" s="2">
         <v>4000</v>
       </c>
-      <c r="B25">
-        <v>90.7</v>
+      <c r="B25" s="2">
+        <v>89.2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26">
+      <c r="A26" s="2">
         <v>5000</v>
       </c>
-      <c r="B26">
-        <v>87.1</v>
+      <c r="B26" s="2">
+        <v>85.6</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27">
+      <c r="A27" s="2">
         <v>6300</v>
       </c>
-      <c r="B27">
-        <v>82.6</v>
+      <c r="B27" s="2">
+        <v>81.099999999999994</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28">
+      <c r="A28" s="2">
         <v>8000</v>
       </c>
-      <c r="B28">
-        <v>77</v>
+      <c r="B28" s="2">
+        <v>75.5</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29">
+      <c r="A29" s="2">
         <v>10000</v>
       </c>
-      <c r="B29">
-        <v>71</v>
+      <c r="B29" s="2">
+        <v>69.5</v>
       </c>
     </row>
   </sheetData>
@@ -645,9 +691,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF0FCF08-DC8C-8747-8876-8E08389E2786}">
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -658,266 +704,258 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2">
-        <v>10</v>
-      </c>
-      <c r="B2">
-        <v>59.9</v>
+      <c r="A2" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="B2" s="4">
+        <v>53.1</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3">
-        <v>12.5</v>
-      </c>
-      <c r="B3">
-        <v>64.7</v>
+      <c r="A3" s="3">
+        <v>16</v>
+      </c>
+      <c r="B3" s="4">
+        <v>58.7</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4">
-        <v>16</v>
-      </c>
-      <c r="B4">
-        <v>69.3</v>
+      <c r="A4" s="3">
+        <v>20</v>
+      </c>
+      <c r="B4" s="4">
+        <v>63.9</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5">
-        <v>20</v>
-      </c>
-      <c r="B5">
+      <c r="A5" s="3">
+        <v>25</v>
+      </c>
+      <c r="B5" s="4">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="3">
+        <v>32</v>
+      </c>
+      <c r="B6" s="4">
         <v>72.599999999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6">
-        <v>25</v>
-      </c>
-      <c r="B6">
+    <row r="7" spans="1:2">
+      <c r="A7" s="3">
+        <v>40</v>
+      </c>
+      <c r="B7" s="4">
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7">
-        <v>31.5</v>
-      </c>
-      <c r="B7">
-        <v>77.900000000000006</v>
-      </c>
-    </row>
     <row r="8" spans="1:2">
-      <c r="A8">
-        <v>40</v>
-      </c>
-      <c r="B8">
+      <c r="A8" s="3">
+        <v>50</v>
+      </c>
+      <c r="B8" s="4">
         <v>79.099999999999994</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9">
-        <v>50</v>
-      </c>
-      <c r="B9">
-        <v>81.099999999999994</v>
+      <c r="A9" s="3">
+        <v>63</v>
+      </c>
+      <c r="B9" s="4">
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10">
-        <v>63</v>
-      </c>
-      <c r="B10">
-        <v>85.4</v>
+      <c r="A10" s="3">
+        <v>80</v>
+      </c>
+      <c r="B10" s="4">
+        <v>84.7</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11">
-        <v>80</v>
-      </c>
-      <c r="B11">
-        <v>88.1</v>
+      <c r="A11" s="3">
+        <v>100</v>
+      </c>
+      <c r="B11" s="4">
+        <v>87.1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12">
-        <v>100</v>
-      </c>
-      <c r="B12">
-        <v>89.7</v>
+      <c r="A12" s="3">
+        <v>125</v>
+      </c>
+      <c r="B12" s="4">
+        <v>89.2</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13">
-        <v>125</v>
-      </c>
-      <c r="B13">
-        <v>92.3</v>
+      <c r="A13" s="3">
+        <v>160</v>
+      </c>
+      <c r="B13" s="4">
+        <v>91.2</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14">
-        <v>160</v>
-      </c>
-      <c r="B14">
-        <v>94.3</v>
+      <c r="A14" s="3">
+        <v>200</v>
+      </c>
+      <c r="B14" s="4">
+        <v>92.7</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15">
-        <v>200</v>
-      </c>
-      <c r="B15">
+      <c r="A15" s="3">
+        <v>250</v>
+      </c>
+      <c r="B15" s="4">
+        <v>93.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="3">
+        <v>315</v>
+      </c>
+      <c r="B16" s="4">
+        <v>93.4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="3">
+        <v>400</v>
+      </c>
+      <c r="B17" s="4">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="3">
+        <v>500</v>
+      </c>
+      <c r="B18" s="4">
+        <v>92.9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="3">
+        <v>630</v>
+      </c>
+      <c r="B19" s="4">
+        <v>93.4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="3">
+        <v>800</v>
+      </c>
+      <c r="B20" s="4">
+        <v>94.4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="3">
+        <v>1000</v>
+      </c>
+      <c r="B21" s="4">
         <v>95.6</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16">
-        <v>250</v>
-      </c>
-      <c r="B16">
+    <row r="22" spans="1:2">
+      <c r="A22" s="3">
+        <v>1250</v>
+      </c>
+      <c r="B22" s="4">
         <v>96.6</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17">
-        <v>315</v>
-      </c>
-      <c r="B17">
-        <v>97.7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18">
-        <v>400</v>
-      </c>
-      <c r="B18">
-        <v>97.8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19">
-        <v>500</v>
-      </c>
-      <c r="B19">
-        <v>97.9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20">
-        <v>630</v>
-      </c>
-      <c r="B20">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21">
-        <v>800</v>
-      </c>
-      <c r="B21">
-        <v>99.8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22">
-        <v>1000</v>
-      </c>
-      <c r="B22">
-        <v>100</v>
-      </c>
-    </row>
     <row r="23" spans="1:2">
-      <c r="A23">
-        <v>1250</v>
-      </c>
-      <c r="B23">
-        <v>100.5</v>
+      <c r="A23" s="3">
+        <v>1600</v>
+      </c>
+      <c r="B23" s="4">
+        <v>97.1</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24">
-        <v>1600</v>
-      </c>
-      <c r="B24">
-        <v>100.3</v>
+      <c r="A24" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B24" s="4">
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25">
-        <v>2000</v>
-      </c>
-      <c r="B25">
-        <v>98.2</v>
+      <c r="A25" s="3">
+        <v>2500</v>
+      </c>
+      <c r="B25" s="4">
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26">
-        <v>2500</v>
-      </c>
-      <c r="B26">
-        <v>94.7</v>
+      <c r="A26" s="3">
+        <v>3150</v>
+      </c>
+      <c r="B26" s="4">
+        <v>93.9</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27">
-        <v>3150</v>
-      </c>
-      <c r="B27">
-        <v>90.4</v>
+      <c r="A27" s="3">
+        <v>4000</v>
+      </c>
+      <c r="B27" s="4">
+        <v>90.5</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28">
-        <v>4000</v>
-      </c>
-      <c r="B28">
-        <v>85.4</v>
+      <c r="A28" s="3">
+        <v>5000</v>
+      </c>
+      <c r="B28" s="4">
+        <v>85.5</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29">
-        <v>5000</v>
-      </c>
-      <c r="B29">
-        <v>80.5</v>
+      <c r="A29" s="3">
+        <v>6300</v>
+      </c>
+      <c r="B29" s="4">
+        <v>79.3</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30">
-        <v>6300</v>
-      </c>
-      <c r="B30">
-        <v>73.400000000000006</v>
+      <c r="A30" s="3">
+        <v>8000</v>
+      </c>
+      <c r="B30" s="4">
+        <v>72.900000000000006</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31">
-        <v>8000</v>
-      </c>
-      <c r="B31">
-        <v>65.7</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32">
+      <c r="A31" s="3">
         <v>10000</v>
       </c>
-      <c r="B32">
-        <v>56.3</v>
+      <c r="B31" s="4">
+        <v>66.5</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -925,42 +963,250 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>63</v>
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>59.9</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>125</v>
+        <v>12.5</v>
+      </c>
+      <c r="B3">
+        <v>64.7</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>250</v>
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>69.3</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>500</v>
+        <v>20</v>
+      </c>
+      <c r="B5">
+        <v>72.599999999999994</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>1000</v>
+        <v>25</v>
+      </c>
+      <c r="B6">
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>2000</v>
+        <v>31.5</v>
+      </c>
+      <c r="B7">
+        <v>77.900000000000006</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>4000</v>
+        <v>40</v>
+      </c>
+      <c r="B8">
+        <v>79.099999999999994</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
+        <v>50</v>
+      </c>
+      <c r="B9">
+        <v>81.099999999999994</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>63</v>
+      </c>
+      <c r="B10">
+        <v>85.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>80</v>
+      </c>
+      <c r="B11">
+        <v>88.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>100</v>
+      </c>
+      <c r="B12">
+        <v>89.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
+        <v>125</v>
+      </c>
+      <c r="B13">
+        <v>92.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <v>160</v>
+      </c>
+      <c r="B14">
+        <v>94.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15">
+        <v>200</v>
+      </c>
+      <c r="B15">
+        <v>95.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16">
+        <v>250</v>
+      </c>
+      <c r="B16">
+        <v>96.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17">
+        <v>315</v>
+      </c>
+      <c r="B17">
+        <v>97.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18">
+        <v>400</v>
+      </c>
+      <c r="B18">
+        <v>97.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19">
+        <v>500</v>
+      </c>
+      <c r="B19">
+        <v>97.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20">
+        <v>630</v>
+      </c>
+      <c r="B20">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21">
+        <v>800</v>
+      </c>
+      <c r="B21">
+        <v>99.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22">
+        <v>1000</v>
+      </c>
+      <c r="B22">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23">
+        <v>1250</v>
+      </c>
+      <c r="B23">
+        <v>100.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24">
+        <v>1600</v>
+      </c>
+      <c r="B24">
+        <v>100.3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25">
+        <v>2000</v>
+      </c>
+      <c r="B25">
+        <v>98.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26">
+        <v>2500</v>
+      </c>
+      <c r="B26">
+        <v>94.7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27">
+        <v>3150</v>
+      </c>
+      <c r="B27">
+        <v>90.4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28">
+        <v>4000</v>
+      </c>
+      <c r="B28">
+        <v>85.4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29">
+        <v>5000</v>
+      </c>
+      <c r="B29">
+        <v>80.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30">
+        <v>6300</v>
+      </c>
+      <c r="B30">
+        <v>73.400000000000006</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31">
         <v>8000</v>
+      </c>
+      <c r="B31">
+        <v>65.7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32">
+        <v>10000</v>
+      </c>
+      <c r="B32">
+        <v>56.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>